<commit_message>
Add cross-track grade comparison and grade-move transfer analysis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016R8Qfohfn7sETBXAmYWCih
</commit_message>
<xml_diff>
--- a/analysis/移籍_格付け表.xlsx
+++ b/analysis/移籍_格付け表.xlsx
@@ -18,9 +18,15 @@
     <sheet name="複勝回収率_変化" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="格の差ごとの集計" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="組み合わせ詳細" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="級の対応表" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="級別の賞金一覧" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="級の移動と成績" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="南関東C級からの移籍" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="級の対応(実績)" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'組み合わせ詳細'!$A$4:$M$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'級の対応(実績)'!$A$4:$F$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +617,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>地方競馬 移籍の格付け表</t>
+          <t>地方競馬 移籍の格付け表・級の比較</t>
         </is>
       </c>
     </row>
@@ -7173,6 +7179,3504 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>各競馬場の級を1着賞金で横並びにした対応表</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>同じ行の級はほぼ同じ賞金水準。重賞・2歳・3歳限定戦は除外。名古屋・笠松の B3〜B12 などは組番号の範囲</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>1着賞金</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>400万〜</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>A2・B1・B2</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr"/>
+      <c r="F5" s="12" t="inlineStr"/>
+      <c r="G5" s="12" t="inlineStr"/>
+      <c r="H5" s="12" t="inlineStr"/>
+      <c r="I5" s="12" t="inlineStr"/>
+      <c r="J5" s="12" t="inlineStr"/>
+      <c r="K5" s="12" t="inlineStr"/>
+      <c r="L5" s="12" t="inlineStr"/>
+      <c r="M5" s="12" t="inlineStr"/>
+      <c r="N5" s="12" t="inlineStr"/>
+      <c r="O5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>250〜399万</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>B1〜B3</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>B1〜B3</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>B1・B2</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr"/>
+      <c r="H6" s="12" t="inlineStr"/>
+      <c r="I6" s="12" t="inlineStr"/>
+      <c r="J6" s="12" t="inlineStr"/>
+      <c r="K6" s="12" t="inlineStr"/>
+      <c r="L6" s="12" t="inlineStr"/>
+      <c r="M6" s="12" t="inlineStr"/>
+      <c r="N6" s="12" t="inlineStr"/>
+      <c r="O6" s="12" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>150〜249万</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr"/>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>A2・B1</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>A級・B1</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr"/>
+      <c r="L7" s="12" t="inlineStr"/>
+      <c r="M7" s="12" t="inlineStr"/>
+      <c r="N7" s="12" t="inlineStr"/>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>100〜149万</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>C1・C2</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>C1・C2</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>B2・C1</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>B2・C1</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>B級</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>A3〜A5</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="N8" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="O8" s="12" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>80〜99万</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr"/>
+      <c r="G9" s="12" t="inlineStr"/>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>A6・B1</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>A3・A4</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="M9" s="12" t="inlineStr"/>
+      <c r="N9" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>A2・A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>60〜79万</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr"/>
+      <c r="C10" s="12" t="inlineStr"/>
+      <c r="D10" s="12" t="inlineStr"/>
+      <c r="E10" s="12" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>C2・C3</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>C2・C3</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>B2〜B12・C1</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>B2〜B4</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="M10" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr"/>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>A4・B1・B2・C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>50〜59万</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr"/>
+      <c r="C11" s="12" t="inlineStr"/>
+      <c r="D11" s="12" t="inlineStr"/>
+      <c r="E11" s="12" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr"/>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr"/>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>C2〜C31</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>C1・C2</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>B1・B2</t>
+        </is>
+      </c>
+      <c r="N11" s="12" t="inlineStr">
+        <is>
+          <t>B級</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>40〜49万</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr"/>
+      <c r="C12" s="12" t="inlineStr"/>
+      <c r="D12" s="12" t="inlineStr"/>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr"/>
+      <c r="G12" s="12" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr"/>
+      <c r="I12" s="12" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>C3・C4</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>C1・C2</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>C1・C2</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>B3〜B10・C2〜C22</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>〜39万</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr"/>
+      <c r="C13" s="12" t="inlineStr"/>
+      <c r="D13" s="12" t="inlineStr"/>
+      <c r="E13" s="12" t="inlineStr"/>
+      <c r="F13" s="12" t="inlineStr"/>
+      <c r="G13" s="12" t="inlineStr"/>
+      <c r="H13" s="12" t="inlineStr"/>
+      <c r="I13" s="12" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr"/>
+      <c r="K13" s="12" t="inlineStr"/>
+      <c r="L13" s="12" t="inlineStr"/>
+      <c r="M13" s="12" t="inlineStr"/>
+      <c r="N13" s="12" t="inlineStr"/>
+      <c r="O13" s="12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>競馬場 × 級 の1着賞金(中央値、万円)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2024年1月〜2026年8月。15レース以上ある級のみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>競馬場</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>級</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>1着賞金中央値(万円)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>レース数</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>620</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>460</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>380</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>大井</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>330</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>船橋</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>500</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>380</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>350</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>浦和</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>川崎</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>320</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>姫路</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>160</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>B級</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>A3〜A4</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>B3〜B12</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>C3〜C23</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>C6〜C31</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>C16〜C30</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D65" s="7" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>B3〜B4</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>C1〜C2</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>C3〜C4</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>A級</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D79" s="7" t="n">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="D81" s="7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D83" s="7" t="n">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="D85" s="7" t="n">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D86" s="7" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="D87" s="7" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>B級</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="D89" s="7" t="n">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D90" s="7" t="n">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D91" s="7" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B92" s="12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="n">
+        <v>95</v>
+      </c>
+      <c r="D92" s="7" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D93" s="7" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D94" s="7" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D95" s="7" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B96" s="12" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D96" s="7" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D97" s="7" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B98" s="12" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B99" s="12" t="inlineStr">
+        <is>
+          <t>B3〜B10</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="D99" s="7" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B100" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B101" s="12" t="inlineStr">
+        <is>
+          <t>C3〜C22</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D101" s="7" t="n">
+        <v>945</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>移籍初戦: 前走の級に対して、移籍先で入った級の賞金水準別の成績</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>比 = 移籍先の級の1着賞金 ÷ 前走の級の1着賞金。回収率は%、人気比1.00=人気どおり</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>級の移動</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>出走数</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>平均人気</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>勝率</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>複勝率</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>単勝回収率</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>複勝回収率</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>人気比</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>大きく下の級(〜0.5倍)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1961</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>44.26</v>
+      </c>
+      <c r="F5" s="28" t="n">
+        <v>73.81999999999999</v>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="H5" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>下の級(0.5〜0.8倍)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>2459</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>95.16</v>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>74.81</v>
+      </c>
+      <c r="H6" s="30" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>同等の級(0.8〜1.2倍)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>2747</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>27.38</v>
+      </c>
+      <c r="F7" s="28" t="n">
+        <v>66.16</v>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>62.58</v>
+      </c>
+      <c r="H7" s="30" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>上の級(1.2〜2倍)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>1662</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>76.31999999999999</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>57.98</v>
+      </c>
+      <c r="H8" s="30" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>大きく上の級(2倍〜)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>503</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="F9" s="28" t="n">
+        <v>52.64</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>61.11</v>
+      </c>
+      <c r="H9" s="30" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>複勝率(%): 級の移動 × 前走着順</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>級の移動</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>前走3着内</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>前走4-6着</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>前走7着以下</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>大きく下の級(〜0.5倍)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>下の級(0.5〜0.8倍)</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>同等の級(0.8〜1.2倍)</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>上の級(1.2〜2倍)</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>大きく上の級(2倍〜)</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B14:D18">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>南関東のC級から他地区へ移籍した馬の初戦成績</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>主な級 = 移籍先で入った級(多い順)。回収率は%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>競馬場</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>出走数</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>主な級</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>移籍先級賞金中央値</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>勝率</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>複勝率</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>平均人気</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>単勝回収率</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>複勝回収率</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>盛岡</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>187</v>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>C2・C1・B2</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H5" s="28" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>81.59999999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>笠松</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>158</v>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>C4・C7・C5</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H6" s="28" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="I6" s="28" t="n">
+        <v>86.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>金沢</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>232</v>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>C2・C1・B2</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>45</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>121.9</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <v>83.59999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>水沢</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>294</v>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>C2・C1・B2</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <v>75.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>佐賀</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>C2・C1・B級</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="n">
+        <v>42</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>93.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>高知</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>135</v>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>C3・C2・C級</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>58.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>門別</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>169</v>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>C4・C3・B3</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H11" s="28" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="I11" s="28" t="n">
+        <v>70.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>288</v>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>B5・B4・B3</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="n">
+        <v>55</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H12" s="28" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="I12" s="28" t="n">
+        <v>52.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>111</v>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>C1・B2・C2</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="n">
+        <v>110</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H13" s="28" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>前走の競馬場・級 → 移籍先の競馬場・級(30件以上)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>実際の移籍で多い級の対応と、移籍初戦の成績</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>元</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>先</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>件数</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>複勝率</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>人気比</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>複勝回収率</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>高知 C3</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>佐賀 C2</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F5" s="28" t="n">
+        <v>99.76000000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>大井 C2</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>浦和 C2</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>22.03</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>106.78</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>高知 C3</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>金沢 C2</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>63.79</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="F7" s="28" t="n">
+        <v>81.72</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>園田 C3</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>佐賀 C2</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>91.88</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>金沢 C2</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>佐賀 C2</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>39.13</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="F9" s="28" t="n">
+        <v>77.17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>門別 C4</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>佐賀 C2</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>44.44</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F10" s="28" t="n">
+        <v>170.67</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>園田 C3</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>金沢 C2</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>41.46</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F11" s="28" t="n">
+        <v>66.83</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>門別 C4</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>園田 C2</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F12" s="28" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>大井 C2</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>船橋 C2</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>30.77</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F13" s="28" t="n">
+        <v>53.08</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>大井 C3</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>浦和 C3</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>46.15</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F14" s="28" t="n">
+        <v>102.05</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>園田 C2</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>佐賀 C2</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>35.14</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F15" s="28" t="n">
+        <v>70.54000000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>大井 C2</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>川崎 C2</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F16" s="28" t="n">
+        <v>49.71</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>門別 C4</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>水沢 C2</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>61.29</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F17" s="28" t="n">
+        <v>126.13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>高知 C3</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>園田 C2</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>19.35</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="F18" s="28" t="n">
+        <v>42.26</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F18"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>